<commit_message>
V2-7a+b: expand card pool (14/9) + multi-level & level-select screen
V2-7a 扩卡池：+6 卡 / +4 单位 → 14 卡 / 9 单位
(mini_pekka/musketeer/skeletons/baby_dragon/lightning/log)，仍走三积木、
不做空地克制；新数值为白膜占位（统一平衡留 V2-8）。Excel 同步 + config_loader 单测。

V2-7b 多关卡 + 选关界面：levels.json 1→4 关（level_01 不动，守旧测试假设）。
新增 EASY 训练场 / HARD 冠军竞技场(含新卡 AI 卡组) / HARD 闪电赛(双倍圣水·120s)，
各关自带 ai_difficulty + AI 卡组 + 塔血 + 圣水节奏。新增 view/level_select 选关界面
（按难度档卡片、从配置动态读取），取代并删除 difficulty_select；难度内嵌进关卡、
经 GameState.level_id 传递；battle_scene 改 setup(GameState.level_id)、难度由关卡解析。
逻辑层零改动（Match/AIController V2-6 已铺好接口）。

文档同步：AGENTS.md（Codex 进度指针，已授权）/ HISTORY.md / CLAUDE.md。
单测 120/120 全过 + headless 烟测（level_03 AI 部署新卡零报错）。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/GameConfig.xlsx
+++ b/config/GameConfig.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Units" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CardSkills" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decks" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance_View" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Enums" sheetId="7" state="hidden" r:id="rId7"/>
+    <sheet name="Units" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cards" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="CardSkills" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Levels" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Decks" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Balance_View" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="_Enums" sheetId="7" state="hidden" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Units'!$A$1:$I$1</definedName>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -664,6 +664,138 @@
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>mini_pekka_body</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>迷你皮卡</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>700</v>
+      </c>
+      <c r="D7" t="n">
+        <v>320</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>musketeer_body</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>火枪手</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>340</v>
+      </c>
+      <c r="D8" t="n">
+        <v>110</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>skeleton_body</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>骷髅</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>40</v>
+      </c>
+      <c r="D9" t="n">
+        <v>40</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>baby_dragon_body</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>小龙</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>900</v>
+      </c>
+      <c r="D10" t="n">
+        <v>80</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>air</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
@@ -682,7 +814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -917,6 +1049,150 @@
       </c>
       <c r="F9" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>mini_pekka</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>迷你皮卡</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>troop</t>
+        </is>
+      </c>
+      <c r="E10" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>musketeer</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>火枪手</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>troop</t>
+        </is>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>skeletons</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>骷髅海</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>troop</t>
+        </is>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>baby_dragon</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>小龙</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>troop</t>
+        </is>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>lightning</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>闪电</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>spell</t>
+        </is>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>log</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>滚木</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>spell</t>
+        </is>
+      </c>
+      <c r="E15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -929,7 +1205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1203,6 +1479,166 @@
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>mini_pekka</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>spawn_unit</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>mini_pekka_body</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>musketeer</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>spawn_unit</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>musketeer_body</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>skeletons</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>spawn_unit</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>skeleton_body</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>baby_dragon</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>spawn_unit</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>baby_dragon_body</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>lightning</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>direct_damage</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="n">
+        <v>280</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>first_enemy_in_lane</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>log</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>aoe_damage</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="n">
+        <v>130</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
@@ -1224,7 +1660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1317,6 +1753,105 @@
         <v>1400</v>
       </c>
       <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>level_02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>训练场</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E3" t="n">
+        <v>180</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1400</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>level_03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>冠军竞技场</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E4" t="n">
+        <v>180</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>2600</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>level_04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>闪电赛</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" t="n">
+        <v>120</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>2400</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1400</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
@@ -1335,7 +1870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1514,6 +2049,324 @@
       </c>
       <c r="K3" t="inlineStr"/>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>level_02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>knight</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>archers</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>giant</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>goblins</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>minions</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>fireball</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>arrows</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>zap</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>level_02</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>knight</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>archers</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>giant</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>goblins</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>minions</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>skeletons</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>arrows</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>zap</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>level_03</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>knight</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>archers</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>giant</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>goblins</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>minions</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>fireball</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>arrows</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>zap</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>level_03</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>giant</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>mini_pekka</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>musketeer</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>baby_dragon</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>minions</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>fireball</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>lightning</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>archers</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>level_04</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>knight</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>archers</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>giant</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>goblins</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>minions</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>fireball</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>arrows</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>zap</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>level_04</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>goblins</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>skeletons</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>knight</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>archers</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>mini_pekka</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>log</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>zap</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>musketeer</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <dataValidations count="1">
@@ -1531,7 +2384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1767,6 +2620,150 @@
         <v>0.06</v>
       </c>
       <c r="I6" t="inlineStr">
+        <is>
+          <t>air</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>mini_pekka_body</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>迷你皮卡</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>700</v>
+      </c>
+      <c r="D7" t="n">
+        <v>320</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F7">
+        <f>IF(E7&gt;0,D7/E7,"")</f>
+        <v/>
+      </c>
+      <c r="G7" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>musketeer_body</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>火枪手</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>340</v>
+      </c>
+      <c r="D8" t="n">
+        <v>110</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F8">
+        <f>IF(E8&gt;0,D8/E8,"")</f>
+        <v/>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>skeleton_body</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>骷髅</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>40</v>
+      </c>
+      <c r="D9" t="n">
+        <v>40</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <f>IF(E9&gt;0,D9/E9,"")</f>
+        <v/>
+      </c>
+      <c r="G9" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>baby_dragon_body</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>小龙</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>900</v>
+      </c>
+      <c r="D10" t="n">
+        <v>80</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F10">
+        <f>IF(E10&gt;0,D10/E10,"")</f>
+        <v/>
+      </c>
+      <c r="G10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>air</t>
         </is>

</xml_diff>

<commit_message>
V2-8: balance pass (light) — arrows→AOE + baby_dragon speedup
纯配置轻量平衡（决策 35）。harness 测量得：节奏健康、难度曲线 proxy
不可读交真人、swarm 不削、baby_dragon 废兵。仅改两张卡：
- arrows: 单体 150@3 → AOE r0.5/140@3（补中号群清；顺带消除对称对局 0-0 僵局）
- baby_dragon_body: 攻速 1.6→1.3（DPS 50→62）
test_skill_system 3 个 direct_damage 用例改指向 lightning；单测 121/121。
Excel 已 --from-json 同步。难度曲线交真人实机验收（清单见 HISTORY V2-8）。

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/GameConfig.xlsx
+++ b/config/GameConfig.xlsx
@@ -782,7 +782,7 @@
         <v>80</v>
       </c>
       <c r="E10" t="n">
-        <v>1.6</v>
+        <v>1.3</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
@@ -1437,20 +1437,18 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>direct_damage</t>
+          <t>aoe_damage</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>150</v>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>first_enemy_in_lane</t>
-        </is>
-      </c>
+        <v>140</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
@@ -2751,7 +2749,7 @@
         <v>80</v>
       </c>
       <c r="E10" t="n">
-        <v>1.6</v>
+        <v>1.3</v>
       </c>
       <c r="F10">
         <f>IF(E10&gt;0,D10/E10,"")</f>

</xml_diff>

<commit_message>
V3-1b: 2D unit movement + flow-field bridge pathfinding (rip-out: delete lane)
推倒重来（决策 37，弃绞杀）：单位从 1D lane 进度重构为 2D 场地坐标，地面兵
沿每塔 BFS 流场梯度自动绕到最近桥过河、逼近敌塔、到攻击距离停下、不踏水。

- unit.gd → 2D（pos:Vector2；move_speed=tile/秒、attack_range=tile）
- arena.gd → units/towers/_flow + build_flow_fields(每塔 BFS) + tick(移动寻路)
- battle.gd → 删 lane(preload/lanes/get_lane/build_v1/build_v2)，step→arena.tick
- skill_system.gd → 2D（原 V3-1f 提前并入）：play_card(card,owner,pos)，aoe 圆/ direct 最近敌
- player.gd → try_play_card(idx,pos) + arena.can_deploy；match.gd → build_arena
- config_loader → attack_range 校验 0~1 改 ≥0
- units.json/cards.json 量纲改 tile；build_config.py 列改名+去 0~1 校验；Excel 同步
- 删 lane.gd + test_lane/test_battle_v2/test_ai_controller；重写 5 测 + arena 移动测
- AI 暂搁置(V3-1g)、view 暂坏(V3-1h)；单测 101/101

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/GameConfig.xlsx
+++ b/config/GameConfig.xlsx
@@ -447,8 +447,8 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
@@ -481,12 +481,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>move_speed_lane_per_s</t>
+          <t>move_speed_tiles_per_s</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>attack_range_lane_ratio</t>
+          <t>attack_range_tiles</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -521,10 +521,10 @@
         <v>1.2</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="G2" t="n">
-        <v>0.05</v>
+        <v>1.2</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -554,10 +554,10 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="G3" t="n">
-        <v>0.25</v>
+        <v>4.5</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -587,10 +587,10 @@
         <v>1.5</v>
       </c>
       <c r="F4" t="n">
-        <v>0.6</v>
+        <v>1.1</v>
       </c>
       <c r="G4" t="n">
-        <v>0.05</v>
+        <v>1.2</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -620,10 +620,10 @@
         <v>1.1</v>
       </c>
       <c r="F5" t="n">
-        <v>1.4</v>
+        <v>2.6</v>
       </c>
       <c r="G5" t="n">
-        <v>0.04</v>
+        <v>1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -653,10 +653,10 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>1.2</v>
+        <v>2.2</v>
       </c>
       <c r="G6" t="n">
-        <v>0.06</v>
+        <v>2</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -686,10 +686,10 @@
         <v>1.8</v>
       </c>
       <c r="F7" t="n">
-        <v>1.1</v>
+        <v>2</v>
       </c>
       <c r="G7" t="n">
-        <v>0.05</v>
+        <v>1.2</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -719,10 +719,10 @@
         <v>1.1</v>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="G8" t="n">
-        <v>0.35</v>
+        <v>5.5</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -752,10 +752,10 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>1.3</v>
+        <v>2.4</v>
       </c>
       <c r="G9" t="n">
-        <v>0.04</v>
+        <v>1</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -785,10 +785,10 @@
         <v>1.3</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="G10" t="n">
-        <v>0.18</v>
+        <v>3</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1421,7 +1421,7 @@
         <v>300</v>
       </c>
       <c r="G7" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
@@ -1446,7 +1446,7 @@
         <v>140</v>
       </c>
       <c r="G8" t="n">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
@@ -1633,7 +1633,7 @@
         <v>130</v>
       </c>
       <c r="G15" t="n">
-        <v>0.4</v>
+        <v>2</v>
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
@@ -2468,10 +2468,10 @@
         <v/>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="H2" t="n">
-        <v>0.05</v>
+        <v>1.2</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -2504,10 +2504,10 @@
         <v/>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="H3" t="n">
-        <v>0.25</v>
+        <v>4.5</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -2540,10 +2540,10 @@
         <v/>
       </c>
       <c r="G4" t="n">
-        <v>0.6</v>
+        <v>1.1</v>
       </c>
       <c r="H4" t="n">
-        <v>0.05</v>
+        <v>1.2</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -2576,10 +2576,10 @@
         <v/>
       </c>
       <c r="G5" t="n">
-        <v>1.4</v>
+        <v>2.6</v>
       </c>
       <c r="H5" t="n">
-        <v>0.04</v>
+        <v>1</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -2612,10 +2612,10 @@
         <v/>
       </c>
       <c r="G6" t="n">
-        <v>1.2</v>
+        <v>2.2</v>
       </c>
       <c r="H6" t="n">
-        <v>0.06</v>
+        <v>2</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -2648,10 +2648,10 @@
         <v/>
       </c>
       <c r="G7" t="n">
-        <v>1.1</v>
+        <v>2</v>
       </c>
       <c r="H7" t="n">
-        <v>0.05</v>
+        <v>1.2</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -2684,10 +2684,10 @@
         <v/>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="H8" t="n">
-        <v>0.35</v>
+        <v>5.5</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -2720,10 +2720,10 @@
         <v/>
       </c>
       <c r="G9" t="n">
-        <v>1.3</v>
+        <v>2.4</v>
       </c>
       <c r="H9" t="n">
-        <v>0.04</v>
+        <v>1</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -2756,10 +2756,10 @@
         <v/>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="H10" t="n">
-        <v>0.18</v>
+        <v>3</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
V3-1c..h: finish 2D combat-core reboot (aggro / collision+attack / tower fire / AI / view)
完成 V3-1 全部子步，lane 模型彻底移除，单测 121/121。
- V3-1c 仇恨/分心：unit +aggro_radius/current_target；arena 索敌(进 aggro 转火直追/否则锁最近敌塔，每 tick 重选回锁)。
- V3-1d 软推挤碰撞 + 接敌攻击：unit +body_radius；arena.tick 五段化(冷却/移动/分离/攻击/清死)；单位能削塔、同 tick 互伤。
- V3-1e 塔会反击：tower +damage/range/attack_speed+冷却；arena 加塔攻击 + 塔毁释放占位重算流场；arena.json +tower_combat。
- V3-1f SkillSystem 2D：已并入 V3-1b（删 lane 连带）。
- V3-1g AIController 2D 重写：2D 部署/威胁/防守空投/集火最弱塔侧/难度分级；test_ai_controller 加回(7 测)。
- V3-1h 显示层 2D：battle_scene 整体重写(tile↔屏幕、地形/河/双桥/6 塔/自由移动单位/塔火/HUD/结算、tap 落点出牌、AI 自驱)。编辑器导入 + 6s headless 实跑零错误；画面/手感待真人验收。
- units.json +aggro_radius/body_radius、build_config.py +两列、Excel 同步 check ok。

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/GameConfig.xlsx
+++ b/config/GameConfig.xlsx
@@ -16,7 +16,7 @@
     <sheet name="_Enums" sheetId="7" state="hidden" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Units'!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Units'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cards'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CardSkills'!$A$1:$I$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Levels'!$A$1:$I$1</definedName>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -449,8 +449,10 @@
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -491,10 +493,20 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>aggro_radius_tiles</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>body_radius_tiles</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>unit_type</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -526,12 +538,18 @@
       <c r="G2" t="n">
         <v>1.2</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>ground</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -559,12 +577,18 @@
       <c r="G3" t="n">
         <v>4.5</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>ground</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -592,12 +616,18 @@
       <c r="G4" t="n">
         <v>1.2</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>ground</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -625,12 +655,18 @@
       <c r="G5" t="n">
         <v>1</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>ground</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -658,12 +694,18 @@
       <c r="G6" t="n">
         <v>2</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>air</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -691,12 +733,18 @@
       <c r="G7" t="n">
         <v>1.2</v>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>ground</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -724,12 +772,18 @@
       <c r="G8" t="n">
         <v>5.5</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H8" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>ground</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -757,12 +811,18 @@
       <c r="G9" t="n">
         <v>1</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J9" t="inlineStr">
         <is>
           <t>ground</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -790,17 +850,23 @@
       <c r="G10" t="n">
         <v>3</v>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H10" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J10" t="inlineStr">
         <is>
           <t>air</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1"/>
+  <autoFilter ref="A1:K1"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ground,air"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
V3-2: air units — flying crosses river + anti-air counter
- unit.gd: +attack_targets(ground/air/both) + is_flying()(=target_type air) + can_hit_type()
- arena.gd: 索敌按 can_hit_type 过滤(纯地面打不到空军/不被其分心)；飞兵 _step_fly 直线越河
  忽略地形；软分离仅同层(空/地互不挤)、_apply_push 飞行可越水/塔。塔不过滤=对空网。
- config/units.json: 每兵 +attack_targets(近战/giant=ground；archer/musketeer/minion/baby_dragon=both)
- tools/build_config.py: +attack_targets 列(ATTACK_TARGETS 枚举+校验+下拉)；Excel 同步
- view/battle_scene.gd: 飞兵上浮 + 地面投影显示
- tests/test_arena.gd: +5(飞兵越水/地面无法对空/对空兵命中/塔对空/空地不互挤)。单测 126/126

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/GameConfig.xlsx
+++ b/config/GameConfig.xlsx
@@ -16,7 +16,7 @@
     <sheet name="_Enums" sheetId="7" state="hidden" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Units'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Units'!$A$1:$L$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cards'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CardSkills'!$A$1:$I$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Levels'!$A$1:$I$1</definedName>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -452,7 +452,8 @@
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -508,6 +509,11 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>attack_targets</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>notes</t>
         </is>
       </c>
@@ -549,7 +555,12 @@
           <t>ground</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -588,7 +599,12 @@
           <t>ground</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -627,7 +643,12 @@
           <t>ground</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -666,7 +687,12 @@
           <t>ground</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -705,7 +731,12 @@
           <t>air</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -744,7 +775,12 @@
           <t>ground</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -783,7 +819,12 @@
           <t>ground</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -822,7 +863,12 @@
           <t>ground</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -861,13 +907,21 @@
           <t>air</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1"/>
-  <dataValidations count="1">
+  <autoFilter ref="A1:L1"/>
+  <dataValidations count="2">
     <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ground,air"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ground,air,both"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
V3-3: new skill blocks — on_death_spawn (golem) + aoe_heal (heal)
数据驱动积木扩展（择优 2 个；slow/击退/建筑留后续）：
- 亡语召唤 on_death_spawn（单位行为）：unit +death_spawn_id/count/config；arena._remove_dead
  死亡裂兵；skill_system 生成时注入 config 模板（arena 不依赖 ConfigLoader）。新卡 golem 死裂 2 哥布林。
- 治疗术 aoe_heal（法术块，复用 radius/damage 列）：unit +heal()；skill_system +_aoe_heal 治友军。新卡 heal。
- config_loader +death_spawn_unit 交叉校验；build_config +aoe_heal/+death_spawn 两列；Excel 同步。
- units.json +golem_body、cards.json +golem/+heal → 16 卡/10 单位。
- tests +3（治友不治敌/治疗封顶/亡语裂兵）。单测 129/129。

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/GameConfig.xlsx
+++ b/config/GameConfig.xlsx
@@ -16,7 +16,7 @@
     <sheet name="_Enums" sheetId="7" state="hidden" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Units'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Units'!$A$1:$N$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cards'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CardSkills'!$A$1:$I$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Levels'!$A$1:$I$1</definedName>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -453,7 +453,9 @@
     <col width="19" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -514,6 +516,16 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>death_spawn_unit</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>death_spawn_count</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>notes</t>
         </is>
       </c>
@@ -561,6 +573,8 @@
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -605,6 +619,8 @@
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -649,6 +665,8 @@
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -693,6 +711,8 @@
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -737,6 +757,8 @@
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -781,6 +803,8 @@
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -825,6 +849,8 @@
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -869,6 +895,8 @@
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -913,9 +941,63 @@
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>golem_body</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>石头人</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D11" t="n">
+        <v>100</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H11" t="n">
+        <v>5</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>goblin_body</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N11" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:N1"/>
   <dataValidations count="2">
     <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ground,air"</formula1>
@@ -934,7 +1016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1313,6 +1395,54 @@
       </c>
       <c r="F15" t="inlineStr"/>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>golem</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>石头人</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>7</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>troop</t>
+        </is>
+      </c>
+      <c r="E16" t="b">
+        <v>1</v>
+      </c>
+      <c r="F16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>heal</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>治疗术</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>spell</t>
+        </is>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1325,7 +1455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1758,11 +1888,63 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>golem</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>spawn_unit</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>golem_body</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>heal</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>aoe_heal</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="n">
+        <v>150</v>
+      </c>
+      <c r="G17" t="n">
+        <v>3</v>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <dataValidations count="2">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"spawn_unit,direct_damage,aoe_damage"</formula1>
+      <formula1>"spawn_unit,direct_damage,aoe_damage,aoe_heal"</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"first_enemy_in_lane"</formula1>
@@ -2502,7 +2684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2887,6 +3069,42 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>golem_body</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>石头人</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D11" t="n">
+        <v>100</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F11">
+        <f>IF(E11&gt;0,D11/E11,"")</f>
+        <v/>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2899,7 +3117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3001,6 +3219,17 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>aoe_heal</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(KAN-80~89): 卡池三维设计 + 三件套引擎(splash/building-target/status) + retrofit + 崩溃修复
- 设计四部曲 docs/design/01-04：16→48 卡稀有度/流派/觉醒三维体系（KAN-80 Done）
- 三件套引擎（KAN-81/82/83，各配单测；客户端 345/345 零回归）：
  - T1 splash: unit.splash_radius + arena._collect_splash（只打单位/尊重对空/排除主目标/确定性）
  - T2 building-target: unit.target_priority + arena._acquire_target 只锁敌塔
  - T3 status: unit 状态计时层 + on_hit_status + 法术 status 块（slow/stun/freeze）
- retrofit（KAN-84）: baby_dragon splash 1.5 / giant·golem 只拆塔；build_config.py 加两列往返同步 xlsx
- 修复（KAN-89）: 闯关进战斗空指针卡死（_ready await 窗口 _process 跑到 null player）
- 真人验收通过：不再崩/卡死 + giant/golem 只拆塔 + baby_dragon(余烬火颅)溅射清群
- KAN-78/79 反作弊实跑 pve_verify pass；运维铁律：改 logic/config 重启 verifier 容器、加卡重启 api

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/GameConfig.xlsx
+++ b/config/GameConfig.xlsx
@@ -16,7 +16,7 @@
     <sheet name="_Enums" sheetId="7" state="hidden" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Units'!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Units'!$A$1:$P$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cards'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CardSkills'!$A$1:$I$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Levels'!$A$1:$I$1</definedName>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -453,9 +453,11 @@
     <col width="19" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="19" customWidth="1" min="13" max="13"/>
-    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -516,15 +518,25 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>splash_radius</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>target_priority</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>death_spawn_unit</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>death_spawn_count</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -575,6 +587,8 @@
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -621,6 +635,8 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -665,8 +681,14 @@
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>buildings</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -713,6 +735,8 @@
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -759,6 +783,8 @@
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -805,6 +831,8 @@
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -851,6 +879,8 @@
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -897,6 +927,8 @@
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -940,9 +972,13 @@
           <t>both</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -986,24 +1022,33 @@
           <t>ground</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>buildings</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
         <is>
           <t>goblin_body</t>
         </is>
       </c>
-      <c r="M11" t="n">
+      <c r="O11" t="n">
         <v>2</v>
       </c>
-      <c r="N11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
-  <dataValidations count="2">
+  <autoFilter ref="A1:P1"/>
+  <dataValidations count="3">
     <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ground,air"</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ground,air,both"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"nearest,buildings"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(KAN-86): epic+legendary signature 觉醒填 rank_unlocks（12 真觉醒 + 4 留 KAN-88）
- 16 张 epic+legendary 填 signature 觉醒（rank3 marquee + rank2 轻量）：
  12 真觉醒用现有 ops+三件套——unit_field 挂 on_hit_status/splash(baby_dragon 烈焰吐息/
  musketeer/wizard/executioner/ice_wizard/princess) + death_spawn(golem 崩解→石心魔像/
  lava_hound 熔火降临/phoenix 重生) + set_field 加 status(lightning 雷暴 stun) +
  num_add(freeze 绝对零度+200伤) + count_add(skeleton_army 亡骨潮)。
  4 留 KAN-88(rank3 stat 占位)：heal haste / balloon T6 death_aoe / electro chain / inferno T7 ramp。
- logic/card_progression.gd +set_field op（设块 field=任意值含嵌套 dict）。
- +2 觉醒专用单位 golemite_body/fire_pup_body；--from-json/--check 往返一致。
- 验证：客户端 353/353（+8 test_v5_awakening）+ rank3 觉醒局重放 smoke 逐 hash 全等 pass；verifier 已重启同步。
- 服务端无改（Go cfg.Cards 忽略 rank_unlocks）。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/GameConfig.xlsx
+++ b/config/GameConfig.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S38"/>
+  <dimension ref="A1:S40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2552,6 +2552,114 @@
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>golemite_body</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>石心魔像</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>400</v>
+      </c>
+      <c r="D39" t="n">
+        <v>40</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H39" t="n">
+        <v>5</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>buildings</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>fire_pup_body</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>喷火火犬</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>110</v>
+      </c>
+      <c r="D40" t="n">
+        <v>40</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F40" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="G40" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H40" t="n">
+        <v>5</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>air</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="L40" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>
@@ -7083,7 +7191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8471,6 +8579,78 @@
         <v>3.5</v>
       </c>
       <c r="I38" t="inlineStr">
+        <is>
+          <t>air</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>golemite_body</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>石心魔像</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>400</v>
+      </c>
+      <c r="D39" t="n">
+        <v>40</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F39">
+        <f>IF(E39&gt;0,D39/E39,"")</f>
+        <v/>
+      </c>
+      <c r="G39" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>fire_pup_body</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>喷火火犬</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>110</v>
+      </c>
+      <c r="D40" t="n">
+        <v>40</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F40">
+        <f>IF(E40&gt;0,D40/E40,"")</f>
+        <v/>
+      </c>
+      <c r="G40" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="H40" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I40" t="inlineStr">
         <is>
           <t>air</t>
         </is>

</xml_diff>